<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-15 20:21 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -701,7 +701,7 @@
     <t>hgutierrez@zitron.com</t>
   </si>
   <si>
-    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ZVN 1-9-75/2,ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB</t>
+    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ZVN 1-9-75/2,ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB,OT4360 -  ZVN 1-9-90/2 + TOB + REJ,OT4360 -  ZVN 1-9-90/2 + TOB + REJ</t>
   </si>
   <si>
     <t>1214046914974309</t>
@@ -5811,7 +5811,7 @@
         <v>46127.69765324074</v>
       </c>
       <c r="D67" s="8">
-        <v>46182.82945164352</v>
+        <v>46188.669512673616</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 19:42 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -7823,7 +7823,7 @@
       </c>
       <c r="C101" s="9"/>
       <c r="D101" s="8">
-        <v>46191.787866087965</v>
+        <v>46192.79300131944</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>323</v>
@@ -8615,7 +8615,7 @@
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46191.78890746528</v>
+        <v>46192.79081532407</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>237</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-21 00:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -7351,7 +7351,7 @@
         <v>46191.77043608796</v>
       </c>
       <c r="D93" s="8">
-        <v>46191.77044953704</v>
+        <v>46193.954018240736</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>303</v>
@@ -7395,8 +7395,8 @@
       <c r="R93" s="8">
         <v>46140</v>
       </c>
-      <c r="S93" s="10" t="s">
-        <v>31</v>
+      <c r="S93" s="12" t="s">
+        <v>122</v>
       </c>
       <c r="T93" s="9">
         <v>1</v>
@@ -7412,9 +7412,11 @@
       <c r="B94" s="5">
         <v>46125.7814462963</v>
       </c>
-      <c r="C94" s="6"/>
+      <c r="C94" s="5">
+        <v>46193.953992442126</v>
+      </c>
       <c r="D94" s="5">
-        <v>46191.768744236106</v>
+        <v>46193.953995034724</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>296</v>
@@ -7465,9 +7467,11 @@
       <c r="B95" s="8">
         <v>46125.78158427084</v>
       </c>
-      <c r="C95" s="9"/>
+      <c r="C95" s="8">
+        <v>46193.95400423611</v>
+      </c>
       <c r="D95" s="8">
-        <v>46191.768768229165</v>
+        <v>46193.9540056713</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>300</v>
@@ -8053,7 +8057,7 @@
       </c>
       <c r="C105" s="9"/>
       <c r="D105" s="8">
-        <v>46148.169578402776</v>
+        <v>46193.95399858797</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>235</v>
@@ -8106,7 +8110,7 @@
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46148.169549467595</v>
+        <v>46193.954008518514</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>237</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 13:43 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -11015,7 +11015,7 @@
       </c>
       <c r="C159" s="9"/>
       <c r="D159" s="8">
-        <v>46195.16796179398</v>
+        <v>46196.17368006945</v>
       </c>
       <c r="E159" s="9" t="s">
         <v>461</v>
@@ -11065,8 +11065,8 @@
       <c r="T159" s="9">
         <v>0</v>
       </c>
-      <c r="U159" s="12" t="s">
-        <v>294</v>
+      <c r="U159" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 22:08 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="8">
-        <v>46133.17089466435</v>
+        <v>46198.87202709491</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>57</v>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46133.17089664352</v>
+        <v>46198.872028495374</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>61</v>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="8">
-        <v>46133.17089804398</v>
+        <v>46198.872029826394</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>64</v>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46133.17089929398</v>
+        <v>46198.87203136574</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>67</v>
@@ -7554,7 +7554,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46191.786592488425</v>
+        <v>46198.87202574074</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>262</v>
@@ -7792,9 +7792,11 @@
       <c r="B100" s="5">
         <v>46077.54519734954</v>
       </c>
-      <c r="C100" s="6"/>
+      <c r="C100" s="5">
+        <v>46198.872020173614</v>
+      </c>
       <c r="D100" s="5">
-        <v>46182.69256461806</v>
+        <v>46198.87203554398</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>58</v>
@@ -7838,11 +7840,11 @@
       <c r="R100" s="5">
         <v>46125</v>
       </c>
-      <c r="S100" s="12" t="s">
-        <v>122</v>
+      <c r="S100" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T100" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U100" s="11" t="s">
         <v>32</v>
@@ -7857,7 +7859,7 @@
       </c>
       <c r="C101" s="9"/>
       <c r="D101" s="8">
-        <v>46198.839731319444</v>
+        <v>46198.87327074074</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>325</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-01 16:38 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -7924,9 +7924,11 @@
       <c r="B102" s="5">
         <v>46125.79029034722</v>
       </c>
-      <c r="C102" s="6"/>
+      <c r="C102" s="5">
+        <v>46204.68543188657</v>
+      </c>
       <c r="D102" s="5">
-        <v>46204.659611875</v>
+        <v>46204.68545116898</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>327</v>
@@ -7970,10 +7972,12 @@
       <c r="R102" s="5">
         <v>46114</v>
       </c>
-      <c r="S102" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="T102" s="6"/>
+      <c r="S102" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="T102" s="6">
+        <v>1</v>
+      </c>
       <c r="U102" s="6"/>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
@@ -8097,7 +8101,7 @@
       </c>
       <c r="C105" s="9"/>
       <c r="D105" s="8">
-        <v>46193.95399858797</v>
+        <v>46204.68543935185</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>235</v>
@@ -8150,7 +8154,7 @@
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46193.954008518514</v>
+        <v>46204.685440601854</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-08 20:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -720,7 +720,7 @@
     <t>gonzalo.davila@zitron.com</t>
   </si>
   <si>
-    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ZVN 1-9-75/2,ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4340 - JZR 6-18.5/2 + 2FAR 60/100 + BASTIDOR,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB,OT4360 -  ZVN 1-9-90/2 + TOB + REJ,OT4360 -  ZVN 1-9-90/2 + TOB + REJ, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2</t>
+    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ZVN 1-9-75/2,ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4340 - JZR 6-18.5/2 + 2FAR 60/100 + BASTIDOR,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB,OT4360 -  ZVN 1-9-90/2 + TOB + REJ,OT4360 -  ZVN 1-9-90/2 + TOB + REJ, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2</t>
   </si>
   <si>
     <t>1214046914974309</t>
@@ -5932,7 +5932,7 @@
         <v>46127.69765324074</v>
       </c>
       <c r="D68" s="5">
-        <v>46209.714337812504</v>
+        <v>46211.815882106486</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>232</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-22 13:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -714,7 +714,7 @@
     <t>gonzalo.davila@zitron.com</t>
   </si>
   <si>
-    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ot 4309- ZVN 1-9-75/2,ot 4309- ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4340 - JZR 6-18.5/2 + 2FAR 60/100 + BASTIDOR,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB,OT4360 -  ZVN 1-9-90/2 + TOB + REJ,OT4360 -  ZVN 1-9-90/2 + TOB + REJ, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2</t>
+    <t>OT 4302 -ZVN 1-10-26/2,OT 4302 -ZVN 1-10-26/2,ot 4309- ZVN 1-9-75/2,ot 4309- ZVN 1-9-75/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2, OT4316  ZVN 1-9-25/4, OT4316  ZVN 1-9-25/4,OT 4317 ZVN 1-16-126/4 ,OT 4313 - ZVN 1-9-45/2,OT 4313 - ZVN 1-9-45/2,OT 4332 -  ZVN 1-16-126/4 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4327- ZVN 2-9-103/2,OT 4327- ZVN 2-9-103/2,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4328 - ZVN 1-9-86/2,OT 4328 - ZVN 1-9-86/2,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4335 - ZVN 1-7-37/2 + TOB + REJ,OT 4340 - JZR 6-18.5/2 + 2FAR 60/100 + BASTIDOR,OT 4342 - ZVN 1-16-160/4 + TOB + REJ + 2FAR 160/200 + TIPO A,OT 4347- ZVN 1-14-75/4 + TIPOC + 2FAR140/200 + TIPOB,OT4360 -  ZVN 1-9-90/2 + TOB + REJ,OT4360 -  ZVN 1-9-90/2 + TOB + REJ, ot 4363 ZVN 1-9-86/2, ot 4363 ZVN 1-9-86/2</t>
   </si>
   <si>
     <t>1214046914974309</t>
@@ -5932,7 +5932,7 @@
         <v>46127.69765324074</v>
       </c>
       <c r="D68" s="5">
-        <v>46211.815882106486</v>
+        <v>46225.017977881944</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>230</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-27 17:19 UTC
</commit_message>
<xml_diff>
--- a/data/50001499 - EQ CHAPARRAL.xlsx
+++ b/data/50001499 - EQ CHAPARRAL.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1910" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="458">
   <si>
     <t>50001499- EQ. CHAPARRAL</t>
   </si>
@@ -8547,7 +8547,7 @@
       </c>
       <c r="C113" s="9"/>
       <c r="D113" s="8">
-        <v>46225.81275493056</v>
+        <v>46230.71153075232</v>
       </c>
       <c r="E113" s="9" t="s">
         <v>352</v>
@@ -8556,9 +8556,11 @@
         <v>26</v>
       </c>
       <c r="G113" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H113" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H113" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I113" s="9"/>
       <c r="J113" s="9"/>
       <c r="K113" s="9" t="s">
@@ -8600,7 +8602,7 @@
         <v>46225.813130532406</v>
       </c>
       <c r="D114" s="5">
-        <v>46225.81313171296</v>
+        <v>46230.711651805555</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>236</v>
@@ -8609,9 +8611,11 @@
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H114" s="6"/>
+        <v>101</v>
+      </c>
+      <c r="H114" s="6" t="s">
+        <v>102</v>
+      </c>
       <c r="I114" s="6"/>
       <c r="J114" s="6"/>
       <c r="K114" s="6" t="s">
@@ -8647,7 +8651,7 @@
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46225.81234634259</v>
+        <v>46230.711765625005</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>240</v>
@@ -8656,9 +8660,11 @@
         <v>26</v>
       </c>
       <c r="G115" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H115" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H115" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I115" s="9"/>
       <c r="J115" s="9"/>
       <c r="K115" s="9" t="s">
@@ -8694,7 +8700,7 @@
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46225.81274479166</v>
+        <v>46230.71188780092</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>356</v>
@@ -8703,9 +8709,11 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H116" s="6"/>
+        <v>101</v>
+      </c>
+      <c r="H116" s="6" t="s">
+        <v>102</v>
+      </c>
       <c r="I116" s="6"/>
       <c r="J116" s="6"/>
       <c r="K116" s="6" t="s">
@@ -8747,7 +8755,7 @@
         <v>46225.813224363425</v>
       </c>
       <c r="D117" s="8">
-        <v>46225.81322589121</v>
+        <v>46230.71219160879</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>236</v>
@@ -8756,9 +8764,11 @@
         <v>26</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H117" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H117" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I117" s="9"/>
       <c r="J117" s="9"/>
       <c r="K117" s="9" t="s">
@@ -8794,7 +8804,7 @@
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46225.81252960648</v>
+        <v>46230.712052268515</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>240</v>
@@ -8803,9 +8813,11 @@
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H118" s="6"/>
+        <v>101</v>
+      </c>
+      <c r="H118" s="6" t="s">
+        <v>102</v>
+      </c>
       <c r="I118" s="6"/>
       <c r="J118" s="6"/>
       <c r="K118" s="6" t="s">
@@ -8841,7 +8853,7 @@
       </c>
       <c r="C119" s="9"/>
       <c r="D119" s="8">
-        <v>46225.81401447917</v>
+        <v>46230.71299550926</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>360</v>
@@ -8850,9 +8862,11 @@
         <v>26</v>
       </c>
       <c r="G119" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H119" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H119" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I119" s="9"/>
       <c r="J119" s="9"/>
       <c r="K119" s="9" t="s">
@@ -8890,7 +8904,7 @@
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46226.82624630787</v>
+        <v>46230.71291037037</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>236</v>
@@ -8899,9 +8913,11 @@
         <v>26</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H120" s="6"/>
+        <v>101</v>
+      </c>
+      <c r="H120" s="6" t="s">
+        <v>102</v>
+      </c>
       <c r="I120" s="6"/>
       <c r="J120" s="6"/>
       <c r="K120" s="6" t="s">
@@ -8937,7 +8953,7 @@
       </c>
       <c r="C121" s="9"/>
       <c r="D121" s="8">
-        <v>46225.81272188657</v>
+        <v>46230.71281320602</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>240</v>
@@ -8946,9 +8962,11 @@
         <v>26</v>
       </c>
       <c r="G121" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H121" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H121" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I121" s="9"/>
       <c r="J121" s="9"/>
       <c r="K121" s="9" t="s">
@@ -9149,7 +9167,7 @@
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="8">
-        <v>46225.8141224537</v>
+        <v>46230.71270855324</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>370</v>
@@ -9158,9 +9176,11 @@
         <v>26</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H125" s="9"/>
+        <v>101</v>
+      </c>
+      <c r="H125" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="I125" s="9"/>
       <c r="J125" s="9"/>
       <c r="K125" s="9" t="s">

</xml_diff>